<commit_message>
Specify QC in annotation
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/27_sn_gila_check/ERCsn_glia_subcluster_info_anno.xlsx
+++ b/processed-data/04_snRNA-seq/27_sn_gila_check/ERCsn_glia_subcluster_info_anno.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/27_sn_gila_check/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/8j/ftgpc01j3vx744_jxfrp_1rc0000gn/T/ch.sudo.cyberduck/editor-2e410720-64de-4a9d-afe0-3aade0a842b4/39743821f4f6107b013628435f237b33/614260095/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{2F8C1C08-9A4D-6044-B8B2-D471674F7BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87AC8A5C-2403-E04D-8AFC-2302CB3A59DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B51FB27-7B9F-424B-B085-152D0E3436FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28500" yWindow="760" windowWidth="27820" windowHeight="21420" xr2:uid="{94B0D7C2-568F-A244-B31E-6B29F3B33498}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="153">
   <si>
     <t>k10</t>
   </si>
@@ -460,9 +460,6 @@
     <t>Vasc.Endo.2</t>
   </si>
   <si>
-    <t>Neuron_ambig</t>
-  </si>
-  <si>
     <t>OPC.5</t>
   </si>
   <si>
@@ -472,14 +469,26 @@
     <t>Vasc.VLMC.4</t>
   </si>
   <si>
-    <t>Macrophage</t>
+    <t>Oligo.Neu.1</t>
+  </si>
+  <si>
+    <t>Oligo.Neu.2</t>
+  </si>
+  <si>
+    <t>Macro</t>
+  </si>
+  <si>
+    <t>cell_type_broad</t>
+  </si>
+  <si>
+    <t>Vasc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -610,6 +619,12 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1334,14 +1349,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BA5E195-4214-724F-A2F9-342B301003E9}">
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1382,7 +1397,7 @@
         <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O1" t="s">
         <v>13</v>
@@ -1393,8 +1408,11 @@
       <c r="Q1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1446,8 +1464,11 @@
       <c r="Q2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1499,8 +1520,11 @@
       <c r="Q3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1552,8 +1576,11 @@
       <c r="Q4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1605,8 +1632,11 @@
       <c r="Q5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1658,8 +1688,11 @@
       <c r="Q6" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1709,10 +1742,13 @@
         <v>94</v>
       </c>
       <c r="Q7" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+      <c r="R7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1764,8 +1800,11 @@
       <c r="Q8" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1817,8 +1856,11 @@
       <c r="Q9" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -1870,8 +1912,11 @@
       <c r="Q10" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1923,8 +1968,11 @@
       <c r="Q11" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1976,8 +2024,11 @@
       <c r="Q12" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -2027,10 +2078,13 @@
         <v>113</v>
       </c>
       <c r="Q13" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+      <c r="R13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -2080,10 +2134,13 @@
         <v>123</v>
       </c>
       <c r="Q14" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+      <c r="R14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2135,8 +2192,11 @@
       <c r="Q15" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -2188,8 +2248,11 @@
       <c r="Q16" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2241,8 +2304,11 @@
       <c r="Q17" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -2294,8 +2360,11 @@
       <c r="Q18" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -2347,8 +2416,11 @@
       <c r="Q19" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -2400,8 +2472,11 @@
       <c r="Q20" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R20" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -2453,8 +2528,11 @@
       <c r="Q21" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>48</v>
       </c>
@@ -2506,8 +2584,11 @@
       <c r="Q22" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -2559,8 +2640,11 @@
       <c r="Q23" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R23" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -2610,10 +2694,13 @@
         <v>118</v>
       </c>
       <c r="Q24" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+      <c r="R24" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -2665,8 +2752,11 @@
       <c r="Q25" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R25" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -2718,8 +2808,11 @@
       <c r="Q26" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -2771,8 +2864,11 @@
       <c r="Q27" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R27" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -2824,8 +2920,11 @@
       <c r="Q28" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R28" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -2877,8 +2976,11 @@
       <c r="Q29" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R29" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>45</v>
       </c>
@@ -2930,8 +3032,11 @@
       <c r="Q30" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R30" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -2983,8 +3088,11 @@
       <c r="Q31" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -3034,10 +3142,13 @@
         <v>56</v>
       </c>
       <c r="Q32" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+      <c r="R32" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -3087,10 +3198,13 @@
         <v>16</v>
       </c>
       <c r="Q33" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+      <c r="R33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -3140,10 +3254,13 @@
         <v>16</v>
       </c>
       <c r="Q34" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="R34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -3193,10 +3310,13 @@
         <v>16</v>
       </c>
       <c r="Q35" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+      <c r="R35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -3246,10 +3366,13 @@
         <v>16</v>
       </c>
       <c r="Q36" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="R36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -3299,10 +3422,13 @@
         <v>16</v>
       </c>
       <c r="Q37" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+      <c r="R37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -3352,10 +3478,13 @@
         <v>16</v>
       </c>
       <c r="Q38" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="R38" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -3405,10 +3534,13 @@
         <v>16</v>
       </c>
       <c r="Q39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+      <c r="R39" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>42</v>
       </c>
@@ -3458,10 +3590,13 @@
         <v>16</v>
       </c>
       <c r="Q40" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+      <c r="R40" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -3511,10 +3646,13 @@
         <v>16</v>
       </c>
       <c r="Q41" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+      <c r="R41" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -3564,7 +3702,10 @@
         <v>16</v>
       </c>
       <c r="Q42" t="s">
-        <v>16</v>
+        <v>126</v>
+      </c>
+      <c r="R42" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -3573,6 +3714,7 @@
       <sortCondition descending="1" ref="C1:C42"/>
     </sortState>
   </autoFilter>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>